<commit_message>
main update for finalization
</commit_message>
<xml_diff>
--- a/inst/example/Attr.Template.xlsx
+++ b/inst/example/Attr.Template.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B12B9F2D-D621-43D8-9283-CC74F3B3E2F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE333942-E3C2-4F4A-A790-3EB051A60D35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5025" yWindow="1440" windowWidth="23505" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Define" sheetId="2" r:id="rId1"/>
@@ -161,12 +161,6 @@
     <t>Flag for type of PK record</t>
   </si>
   <si>
-    <t>1=300 mg theoph form 1
-2=300 mg theoph form 2
-3=600 mg theoph form 1
-4=1200 mg theoph form 1</t>
-  </si>
-  <si>
     <t>1=Dosing compartment
 2=Central compartment</t>
   </si>
@@ -202,6 +196,11 @@
   </si>
   <si>
     <t>Original dose units set to mg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1=300 mg theoph form 1
+2=300 mg theoph form 2
+</t>
   </si>
 </sst>
 </file>
@@ -327,7 +326,7 @@
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>600075</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>47624</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -877,7 +876,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="5" customWidth="1"/>
@@ -906,7 +905,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -931,7 +930,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -942,7 +941,7 @@
         <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -956,7 +955,7 @@
         <v>11</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -970,7 +969,7 @@
         <v>35</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -978,10 +977,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -989,10 +988,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1000,10 +999,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1011,24 +1010,21 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -1036,52 +1032,55 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C13" t="s">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>39</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1089,10 +1088,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C16" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1100,10 +1099,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" t="s">
         <v>46</v>
-      </c>
-      <c r="C17" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1111,39 +1110,36 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="C18" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C19" t="s">
-        <v>40</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="C20" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21"/>
+        <v>40</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22"/>
@@ -1180,7 +1176,6 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33"/>
-      <c r="F33" s="6"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34"/>
@@ -1188,6 +1183,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35"/>
+      <c r="F35" s="6"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36"/>
@@ -1201,15 +1197,12 @@
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39"/>
     </row>
-    <row r="40" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40"/>
-      <c r="E40" s="7"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" t="e">
-        <f>IF(#REF!=1,SUM(#REF!),"")</f>
-        <v>#REF!</v>
-      </c>
+    </row>
+    <row r="41" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41"/>
+      <c r="E41" s="7"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="e">
@@ -1222,22 +1215,22 @@
         <f>IF(#REF!=1,SUM(#REF!),"")</f>
         <v>#REF!</v>
       </c>
-      <c r="F45" s="8"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="e">
         <f>IF(#REF!=1,SUM(#REF!),"")</f>
         <v>#REF!</v>
       </c>
+      <c r="F46" s="8"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" t="e">
+      <c r="A47" t="e">
         <f>IF(#REF!=1,SUM(#REF!),"")</f>
         <v>#REF!</v>
       </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="e">
@@ -1277,6 +1270,12 @@
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="e">
+        <f>IF(#REF!=1,SUM(#REF!),"")</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="e">
         <f>IF(#REF!=1,SUM(#REF!),"")</f>
         <v>#REF!</v>
       </c>

</xml_diff>